<commit_message>
Add district field readiness checks
</commit_message>
<xml_diff>
--- a/sample_data/orders_sample.xlsx
+++ b/sample_data/orders_sample.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD3"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -532,40 +532,45 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
+          <t>区县</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>发货时间</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>成本</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>快递费</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>物流费</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>运费</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>辅料</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>分摊费用</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>利润</t>
         </is>
@@ -674,29 +679,34 @@
           <t>杭州</t>
         </is>
       </c>
-      <c r="W2" s="1" t="n">
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>余杭区</t>
+        </is>
+      </c>
+      <c r="X2" s="1" t="n">
         <v>46204.4375</v>
       </c>
-      <c r="X2" t="n">
+      <c r="Y2" t="n">
         <v>92</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="Z2" t="n">
         <v>12</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AA2" t="n">
         <v>0</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AB2" t="n">
         <v>8</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AC2" t="n">
         <v>3</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AD2" t="n">
         <v>5</v>
       </c>
-      <c r="AD2" t="n">
-        <v>78</v>
+      <c r="AE2" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="3">
@@ -802,29 +812,34 @@
           <t>广州</t>
         </is>
       </c>
-      <c r="W3" s="1" t="n">
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>天河区</t>
+        </is>
+      </c>
+      <c r="X3" s="1" t="n">
         <v>46205.625</v>
       </c>
-      <c r="X3" t="n">
+      <c r="Y3" t="n">
         <v>125</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="Z3" t="n">
         <v>20</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AA3" t="n">
         <v>5</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AB3" t="n">
         <v>10</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AC3" t="n">
         <v>8</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AD3" t="n">
         <v>7</v>
       </c>
-      <c r="AD3" t="n">
-        <v>70</v>
+      <c r="AE3" t="n">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update import template and receiver address
</commit_message>
<xml_diff>
--- a/sample_data/orders_sample.xlsx
+++ b/sample_data/orders_sample.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AF3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,17 +447,17 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>部门</t>
+          <t>渠道分类</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>平台渠道</t>
+          <t>渠道平台</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>店铺</t>
+          <t>销售渠道</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
@@ -467,12 +467,12 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>原始单号</t>
+          <t>网店订单号（新）</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>物流方式</t>
+          <t>物流公司</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -487,90 +487,95 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>地址</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>电话</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>大类</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>产品名称</t>
-        </is>
-      </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>货品名称</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>货品编号</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>单位</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>数量</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>应收合计分摊</t>
-        </is>
-      </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>州省</t>
+          <t>销售额</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>区市</t>
+          <t>省</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>区县</t>
+          <t>市</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>县</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
           <t>发货时间</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>成本</t>
-        </is>
-      </c>
       <c r="Z1" t="inlineStr">
         <is>
+          <t>成本金额</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
           <t>快递费</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>物流费</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>运费</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>辅料</t>
-        </is>
-      </c>
       <c r="AD1" t="inlineStr">
         <is>
+          <t>辅料费用</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>分摊费用</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>利润</t>
         </is>
@@ -640,72 +645,77 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>浙江省杭州市余杭区未来科技城示例路 1 号</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>13800000001</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>家居</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>收纳箱 45L</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>P-BOX-45</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>个</t>
         </is>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>2</v>
       </c>
-      <c r="T2" t="n">
+      <c r="U2" t="n">
         <v>198</v>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>浙江</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>杭州</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>余杭区</t>
         </is>
       </c>
-      <c r="X2" s="1" t="n">
+      <c r="Y2" s="1" t="n">
         <v>46204.4375</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="Z2" t="n">
         <v>92</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AA2" t="n">
         <v>12</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AB2" t="n">
         <v>0</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AC2" t="n">
         <v>8</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AD2" t="n">
         <v>3</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="AE2" t="n">
         <v>5</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="AF2" t="n">
         <v>90</v>
       </c>
     </row>
@@ -773,72 +783,77 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
+          <t>广东省广州市天河区珠江新城示例路 2 号</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
           <t>13900000002</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>个护</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>旅行洗漱包</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>P-BAG-01</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>个</t>
         </is>
       </c>
-      <c r="S3" t="n">
+      <c r="T3" t="n">
         <v>5</v>
       </c>
-      <c r="T3" t="n">
+      <c r="U3" t="n">
         <v>245</v>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>广东</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>广州</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>天河区</t>
         </is>
       </c>
-      <c r="X3" s="1" t="n">
+      <c r="Y3" s="1" t="n">
         <v>46205.625</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="Z3" t="n">
         <v>125</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AA3" t="n">
         <v>20</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AB3" t="n">
         <v>5</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AC3" t="n">
         <v>10</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AD3" t="n">
         <v>8</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="AE3" t="n">
         <v>7</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AF3" t="n">
         <v>95</v>
       </c>
     </row>

</xml_diff>